<commit_message>
Added files for updated manuscript
-Updated models
-Updated training scripts
-Updated analyses
</commit_message>
<xml_diff>
--- a/Data_Generation_and_Simulation/Models_and_Constraints/GlyPPP_Constraints1of3_20pct.xlsx
+++ b/Data_Generation_and_Simulation/Models_and_Constraints/GlyPPP_Constraints1of3_20pct.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/richardlaw/Library/CloudStorage/Box-Box/ML-Flux/Data/GlyPPP/Constraints/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/860814577223918d/Documents/GitHub/MLFlux/model/MetabolicNetworksAndConstraints/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D40980A-320F-4444-816F-3A9205BE5FB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="13_ncr:1_{3D40980A-320F-4444-816F-3A9205BE5FB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{60E445B9-27A5-4EC6-8B09-16D19D48988C}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="24500" windowHeight="28300" activeTab="2" xr2:uid="{97E65C2A-E213-46AE-9CAD-229F2787D374}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{97E65C2A-E213-46AE-9CAD-229F2787D374}"/>
   </bookViews>
   <sheets>
     <sheet name="net" sheetId="1" r:id="rId1"/>
@@ -200,6 +200,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -500,13 +504,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49FFD124-A179-4710-8E46-0DF171EEF42F}">
   <dimension ref="A1:C35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -517,7 +521,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>490</v>
       </c>
@@ -528,7 +532,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -539,7 +543,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>990</v>
       </c>
@@ -550,7 +554,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -561,7 +565,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>90</v>
       </c>
@@ -572,7 +576,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -583,7 +587,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>90</v>
       </c>
@@ -594,7 +598,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -605,9 +609,9 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="B10" t="s">
         <v>0</v>
@@ -616,7 +620,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -624,10 +628,10 @@
         <v>0</v>
       </c>
       <c r="C11">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>0</v>
       </c>
@@ -635,10 +639,10 @@
         <v>0</v>
       </c>
       <c r="C12" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -649,7 +653,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>0</v>
       </c>
@@ -660,7 +664,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>9</v>
       </c>
@@ -671,7 +675,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>490</v>
       </c>
@@ -682,7 +686,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>10</v>
       </c>
@@ -693,7 +697,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>990</v>
       </c>
@@ -704,7 +708,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>11</v>
       </c>
@@ -715,7 +719,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>90</v>
       </c>
@@ -726,7 +730,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>12</v>
       </c>
@@ -737,7 +741,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>90</v>
       </c>
@@ -748,7 +752,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>13</v>
       </c>
@@ -759,7 +763,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>0.01</v>
       </c>
@@ -770,7 +774,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>14</v>
       </c>
@@ -781,7 +785,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>0.01</v>
       </c>
@@ -792,7 +796,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>15</v>
       </c>
@@ -803,7 +807,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>0.01</v>
       </c>
@@ -814,7 +818,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>16</v>
       </c>
@@ -825,7 +829,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>0.01</v>
       </c>
@@ -836,7 +840,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>17</v>
       </c>
@@ -847,7 +851,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>0.01</v>
       </c>
@@ -858,7 +862,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>18</v>
       </c>
@@ -869,7 +873,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>0.01</v>
       </c>
@@ -880,7 +884,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>0.01</v>
       </c>
@@ -899,9 +903,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30C868E3-6BA7-7A46-91B7-92C782FEF366}">
   <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -920,13 +924,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0087E4DC-7BF1-43BF-88C3-6F205D54E558}">
   <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -937,7 +941,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>20</v>
       </c>
@@ -948,7 +952,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -959,7 +963,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -970,7 +974,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>23</v>
       </c>
@@ -981,7 +985,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -992,7 +996,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -1003,7 +1007,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>26</v>
       </c>
@@ -1014,7 +1018,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>27</v>
       </c>
@@ -1022,10 +1026,10 @@
         <v>0</v>
       </c>
       <c r="C9">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>28</v>
       </c>
@@ -1033,10 +1037,10 @@
         <v>0</v>
       </c>
       <c r="C10">
-        <v>0.01</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>29</v>
       </c>
@@ -1044,10 +1048,10 @@
         <v>0</v>
       </c>
       <c r="C11">
-        <v>0.01</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>30</v>
       </c>
@@ -1055,10 +1059,10 @@
         <v>0</v>
       </c>
       <c r="C12">
-        <v>0.01</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -1066,10 +1070,10 @@
         <v>0</v>
       </c>
       <c r="C13">
-        <v>0.01</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -1077,10 +1081,10 @@
         <v>0</v>
       </c>
       <c r="C14">
-        <v>0.01</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>33</v>
       </c>
@@ -1088,7 +1092,7 @@
         <v>0</v>
       </c>
       <c r="C15">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
     </row>
   </sheetData>
@@ -1099,9 +1103,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{635600A8-6ACB-AE4D-8E15-F81685A703A5}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>7</v>
       </c>
@@ -1112,7 +1116,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -1123,7 +1127,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>

</xml_diff>